<commit_message>
feat(testing): update Appium E2E test suite to include logout verification and robust selectors
</commit_message>
<xml_diff>
--- a/backend/testing/selenium-tests/test_report.xlsx
+++ b/backend/testing/selenium-tests/test_report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="182">
   <si>
     <t>Metric</t>
   </si>
@@ -29,7 +29,7 @@
     <t>Test Execution Date</t>
   </si>
   <si>
-    <t>16/6/2026, 11:18:03 am</t>
+    <t>16/6/2026, 5:16:49 pm</t>
   </si>
   <si>
     <t>Total Steps Executed</t>
@@ -74,7 +74,7 @@
     <t>PASSED</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:51.672Z</t>
+    <t>2026-06-16T11:46:36.753Z</t>
   </si>
   <si>
     <t>Static server hosted successfully</t>
@@ -83,7 +83,7 @@
     <t>WebDriver Session Initialization</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:52.717Z</t>
+    <t>2026-06-16T11:46:38.784Z</t>
   </si>
   <si>
     <t>Chrome headless instance created</t>
@@ -92,7 +92,7 @@
     <t>Load Application URL</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:53.166Z</t>
+    <t>2026-06-16T11:46:39.281Z</t>
   </si>
   <si>
     <t>Target loaded at http://localhost:8095</t>
@@ -101,7 +101,7 @@
     <t>Check Flutter Canvas Elements</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:53.852Z</t>
+    <t>2026-06-16T11:46:40.451Z</t>
   </si>
   <si>
     <t>Glass pane initialized in DOM</t>
@@ -110,7 +110,7 @@
     <t>Enable Web Accessibility Semantics</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:53.855Z</t>
+    <t>2026-06-16T11:46:40.464Z</t>
   </si>
   <si>
     <t>Accessibility tree configured: SUCCESS</t>
@@ -119,7 +119,7 @@
     <t>Verify Slide 1: Welcome Screen Text</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:58.254Z</t>
+    <t>2026-06-16T11:46:45.007Z</t>
   </si>
   <si>
     <t>Main onboarding welcome text verified</t>
@@ -128,7 +128,7 @@
     <t>Verify Onboarding Pagination Dots</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:58.307Z</t>
+    <t>2026-06-16T11:46:45.026Z</t>
   </si>
   <si>
     <t>Skip overlay controls are interactable</t>
@@ -137,7 +137,7 @@
     <t>Verify Skip Button Interactive Bounds</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:58.345Z</t>
+    <t>2026-06-16T11:46:45.034Z</t>
   </si>
   <si>
     <t>Skip action element verified in semantics tree</t>
@@ -146,7 +146,7 @@
     <t>Perform Skip Redirection Transition</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:58.740Z</t>
+    <t>2026-06-16T11:46:45.542Z</t>
   </si>
   <si>
     <t>Redirection to auth screen verified</t>
@@ -155,7 +155,7 @@
     <t>Verify Sign In Heading Presence</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:58.758Z</t>
+    <t>2026-06-16T11:46:45.607Z</t>
   </si>
   <si>
     <t>Login branding header located</t>
@@ -164,7 +164,7 @@
     <t>Submit Blank Form to Verify Inputs</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:59.784Z</t>
+    <t>2026-06-16T11:46:46.689Z</t>
   </si>
   <si>
     <t>Submitted empty credentials form</t>
@@ -173,7 +173,7 @@
     <t>Check Validation Warn: Email Missing</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:59.801Z</t>
+    <t>2026-06-16T11:46:46.704Z</t>
   </si>
   <si>
     <t>Blank validation triggers correct warning</t>
@@ -182,7 +182,7 @@
     <t>Inject Malformed Username Format</t>
   </si>
   <si>
-    <t>2026-06-16T05:47:59.821Z</t>
+    <t>2026-06-16T11:46:46.750Z</t>
   </si>
   <si>
     <t>Typed invalid format string</t>
@@ -191,7 +191,7 @@
     <t>Submit Credentials Payload</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:02.869Z</t>
+    <t>2026-06-16T11:46:49.835Z</t>
   </si>
   <si>
     <t>Dispatched validation credentials</t>
@@ -200,7 +200,7 @@
     <t>Functional UI Validation: Browser Viewport: Width is positive (Assert #1)</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:02.889Z</t>
+    <t>2026-06-16T11:46:49.851Z</t>
   </si>
   <si>
     <t>Width: 1258px</t>
@@ -239,15 +239,15 @@
     <t>Functional UI Validation: Browser Viewport: Document state is ready/complete (Assert #7)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.852Z</t>
+  </si>
+  <si>
     <t>ReadyState: complete</t>
   </si>
   <si>
     <t>Functional UI Validation: Browser Viewport: Local Storage API is available (Assert #8)</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:02.890Z</t>
-  </si>
-  <si>
     <t>UI element attribute verification passed successfully</t>
   </si>
   <si>
@@ -326,6 +326,9 @@
     <t>Functional UI Validation: Authentication Form: Document Character Set is UTF-8 (Assert #23)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.853Z</t>
+  </si>
+  <si>
     <t>CharSet: UTF-8</t>
   </si>
   <si>
@@ -380,12 +383,18 @@
     <t>Functional UI Validation: Browser Viewport: Cookies support is active (Assert #34)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.854Z</t>
+  </si>
+  <si>
     <t>Functional UI Validation: Browser Viewport: User preferred language is set (Assert #35)</t>
   </si>
   <si>
     <t>Functional UI Validation: Browser Viewport: Document state is ready/complete (Assert #36)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.855Z</t>
+  </si>
+  <si>
     <t>Functional UI Validation: Browser Viewport: Local Storage API is available (Assert #37)</t>
   </si>
   <si>
@@ -425,9 +434,6 @@
     <t>Functional UI Validation: Accessibility Engine: Semantics host is not hidden via CSS (Assert #49)</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:02.891Z</t>
-  </si>
-  <si>
     <t>Functional UI Validation: Accessibility Engine: Semantics tree contains nodes (Assert #50)</t>
   </si>
   <si>
@@ -479,6 +485,9 @@
     <t>Functional UI Validation: Browser Viewport: Local Storage API is available (Assert #66)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.856Z</t>
+  </si>
+  <si>
     <t>Functional UI Validation: Browser Viewport: Session Storage API is available (Assert #67)</t>
   </si>
   <si>
@@ -506,6 +515,9 @@
     <t>Functional UI Validation: Glass Pane Container: CSS visibility is visible (Assert #75)</t>
   </si>
   <si>
+    <t>2026-06-16T11:46:49.857Z</t>
+  </si>
+  <si>
     <t>Functional UI Validation: Glass Pane Container: CSS opacity matches default visibility (Assert #76)</t>
   </si>
   <si>
@@ -515,9 +527,6 @@
     <t>Functional UI Validation: Accessibility Engine: Semantics host is not hidden via CSS (Assert #78)</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:02.892Z</t>
-  </si>
-  <si>
     <t>Functional UI Validation: Accessibility Engine: Semantics tree contains nodes (Assert #79)</t>
   </si>
   <si>
@@ -545,7 +554,7 @@
     <t>Shutdown Browser &amp; Terminate Server</t>
   </si>
   <si>
-    <t>2026-06-16T05:48:03.257Z</t>
+    <t>2026-06-16T11:46:49.987Z</t>
   </si>
   <si>
     <t>All background processes killed cleanly</t>
@@ -1048,7 +1057,7 @@
         <v>11</v>
       </c>
       <c r="B8" s="3">
-        <v>13.85</v>
+        <v>13.5</v>
       </c>
     </row>
   </sheetData>
@@ -1100,7 +1109,7 @@
         <v>19</v>
       </c>
       <c r="D2" s="9">
-        <v>2017</v>
+        <v>6</v>
       </c>
       <c r="E2" t="s">
         <v>20</v>
@@ -1120,7 +1129,7 @@
         <v>19</v>
       </c>
       <c r="D3" s="9">
-        <v>1045</v>
+        <v>2030</v>
       </c>
       <c r="E3" t="s">
         <v>23</v>
@@ -1140,7 +1149,7 @@
         <v>19</v>
       </c>
       <c r="D4" s="9">
-        <v>449</v>
+        <v>497</v>
       </c>
       <c r="E4" t="s">
         <v>26</v>
@@ -1160,7 +1169,7 @@
         <v>19</v>
       </c>
       <c r="D5" s="9">
-        <v>686</v>
+        <v>1170</v>
       </c>
       <c r="E5" t="s">
         <v>29</v>
@@ -1180,7 +1189,7 @@
         <v>19</v>
       </c>
       <c r="D6" s="9">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
         <v>32</v>
@@ -1200,7 +1209,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="9">
-        <v>4399</v>
+        <v>4543</v>
       </c>
       <c r="E7" t="s">
         <v>35</v>
@@ -1220,7 +1229,7 @@
         <v>19</v>
       </c>
       <c r="D8" s="9">
-        <v>52</v>
+        <v>19</v>
       </c>
       <c r="E8" t="s">
         <v>38</v>
@@ -1240,7 +1249,7 @@
         <v>19</v>
       </c>
       <c r="D9" s="9">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="E9" t="s">
         <v>41</v>
@@ -1260,7 +1269,7 @@
         <v>19</v>
       </c>
       <c r="D10" s="9">
-        <v>395</v>
+        <v>508</v>
       </c>
       <c r="E10" t="s">
         <v>44</v>
@@ -1280,7 +1289,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="9">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
         <v>47</v>
@@ -1300,7 +1309,7 @@
         <v>19</v>
       </c>
       <c r="D12" s="9">
-        <v>1026</v>
+        <v>1081</v>
       </c>
       <c r="E12" t="s">
         <v>50</v>
@@ -1320,7 +1329,7 @@
         <v>19</v>
       </c>
       <c r="D13" s="9">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E13" t="s">
         <v>53</v>
@@ -1340,7 +1349,7 @@
         <v>19</v>
       </c>
       <c r="D14" s="9">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E14" t="s">
         <v>56</v>
@@ -1360,7 +1369,7 @@
         <v>19</v>
       </c>
       <c r="D15" s="9">
-        <v>3048</v>
+        <v>3085</v>
       </c>
       <c r="E15" t="s">
         <v>59</v>
@@ -1380,7 +1389,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E16" t="s">
         <v>62</v>
@@ -1440,7 +1449,7 @@
         <v>19</v>
       </c>
       <c r="D19" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E19" t="s">
         <v>62</v>
@@ -1460,7 +1469,7 @@
         <v>19</v>
       </c>
       <c r="D20" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E20" t="s">
         <v>62</v>
@@ -1480,7 +1489,7 @@
         <v>19</v>
       </c>
       <c r="D21" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E21" t="s">
         <v>62</v>
@@ -1500,13 +1509,13 @@
         <v>19</v>
       </c>
       <c r="D22" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
       <c r="F22" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -1514,16 +1523,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F23" t="s">
         <v>78</v>
@@ -1540,10 +1549,10 @@
         <v>19</v>
       </c>
       <c r="D24" s="9">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E24" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F24" t="s">
         <v>78</v>
@@ -1563,7 +1572,7 @@
         <v>2</v>
       </c>
       <c r="E25" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F25" t="s">
         <v>81</v>
@@ -1583,7 +1592,7 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F26" t="s">
         <v>83</v>
@@ -1600,10 +1609,10 @@
         <v>19</v>
       </c>
       <c r="D27" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F27" t="s">
         <v>85</v>
@@ -1620,10 +1629,10 @@
         <v>19</v>
       </c>
       <c r="D28" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F28" t="s">
         <v>87</v>
@@ -1640,10 +1649,10 @@
         <v>19</v>
       </c>
       <c r="D29" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F29" t="s">
         <v>89</v>
@@ -1660,10 +1669,10 @@
         <v>19</v>
       </c>
       <c r="D30" s="9">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E30" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F30" t="s">
         <v>78</v>
@@ -1683,7 +1692,7 @@
         <v>2</v>
       </c>
       <c r="E31" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F31" t="s">
         <v>92</v>
@@ -1700,10 +1709,10 @@
         <v>19</v>
       </c>
       <c r="D32" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E32" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F32" t="s">
         <v>94</v>
@@ -1720,10 +1729,10 @@
         <v>19</v>
       </c>
       <c r="D33" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F33" t="s">
         <v>96</v>
@@ -1740,10 +1749,10 @@
         <v>19</v>
       </c>
       <c r="D34" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E34" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F34" t="s">
         <v>78</v>
@@ -1760,10 +1769,10 @@
         <v>19</v>
       </c>
       <c r="D35" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F35" t="s">
         <v>78</v>
@@ -1780,10 +1789,10 @@
         <v>19</v>
       </c>
       <c r="D36" s="9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F36" t="s">
         <v>100</v>
@@ -1800,10 +1809,10 @@
         <v>19</v>
       </c>
       <c r="D37" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F37" t="s">
         <v>102</v>
@@ -1820,13 +1829,13 @@
         <v>19</v>
       </c>
       <c r="D38" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F38" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -1834,19 +1843,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D39" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E39" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F39" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -1854,19 +1863,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D40" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F40" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -1874,7 +1883,7 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>19</v>
@@ -1883,10 +1892,10 @@
         <v>5</v>
       </c>
       <c r="E41" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F41" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -1894,19 +1903,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D42" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E42" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F42" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1914,19 +1923,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D43" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E43" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F43" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -1934,19 +1943,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D44" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E44" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F44" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -1954,16 +1963,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D45" s="9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E45" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F45" t="s">
         <v>63</v>
@@ -1974,16 +1983,16 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C46" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D46" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E46" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F46" t="s">
         <v>65</v>
@@ -1994,16 +2003,16 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C47" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D47" s="9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F47" t="s">
         <v>67</v>
@@ -2014,16 +2023,16 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C48" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D48" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E48" t="s">
-        <v>77</v>
+        <v>104</v>
       </c>
       <c r="F48" t="s">
         <v>69</v>
@@ -2034,16 +2043,16 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C49" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D49" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E49" t="s">
-        <v>77</v>
+        <v>123</v>
       </c>
       <c r="F49" t="s">
         <v>71</v>
@@ -2054,16 +2063,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C50" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D50" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E50" t="s">
-        <v>77</v>
+        <v>123</v>
       </c>
       <c r="F50" t="s">
         <v>73</v>
@@ -2074,19 +2083,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C51" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D51" s="9">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E51" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F51" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -2094,7 +2103,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C52" s="8" t="s">
         <v>19</v>
@@ -2103,7 +2112,7 @@
         <v>3</v>
       </c>
       <c r="E52" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F52" t="s">
         <v>78</v>
@@ -2114,7 +2123,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C53" s="8" t="s">
         <v>19</v>
@@ -2123,7 +2132,7 @@
         <v>2</v>
       </c>
       <c r="E53" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F53" t="s">
         <v>78</v>
@@ -2134,16 +2143,16 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C54" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D54" s="9">
+        <v>2</v>
+      </c>
+      <c r="E54" t="s">
         <v>126</v>
-      </c>
-      <c r="C54" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D54" s="9">
-        <v>4</v>
-      </c>
-      <c r="E54" t="s">
-        <v>77</v>
       </c>
       <c r="F54" t="s">
         <v>81</v>
@@ -2154,16 +2163,16 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D55" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E55" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F55" t="s">
         <v>83</v>
@@ -2174,16 +2183,16 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D56" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E56" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F56" t="s">
         <v>85</v>
@@ -2194,16 +2203,16 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D57" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E57" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F57" t="s">
         <v>87</v>
@@ -2214,16 +2223,16 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D58" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E58" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F58" t="s">
         <v>89</v>
@@ -2234,16 +2243,16 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D59" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E59" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F59" t="s">
         <v>78</v>
@@ -2254,16 +2263,16 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D60" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E60" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F60" t="s">
         <v>92</v>
@@ -2274,7 +2283,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>19</v>
@@ -2283,7 +2292,7 @@
         <v>1</v>
       </c>
       <c r="E61" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F61" t="s">
         <v>94</v>
@@ -2294,16 +2303,16 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D62" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E62" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F62" t="s">
         <v>96</v>
@@ -2314,16 +2323,16 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D63" s="9">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E63" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="F63" t="s">
         <v>78</v>
@@ -2334,16 +2343,16 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D64" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E64" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F64" t="s">
         <v>78</v>
@@ -2354,16 +2363,16 @@
         <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D65" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E65" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F65" t="s">
         <v>100</v>
@@ -2374,16 +2383,16 @@
         <v>65</v>
       </c>
       <c r="B66" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D66" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E66" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F66" t="s">
         <v>102</v>
@@ -2394,7 +2403,7 @@
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>19</v>
@@ -2403,10 +2412,10 @@
         <v>3</v>
       </c>
       <c r="E67" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F67" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2414,7 +2423,7 @@
         <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C68" s="8" t="s">
         <v>19</v>
@@ -2423,10 +2432,10 @@
         <v>4</v>
       </c>
       <c r="E68" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F68" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -2434,19 +2443,19 @@
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C69" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D69" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E69" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F69" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -2454,7 +2463,7 @@
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C70" s="8" t="s">
         <v>19</v>
@@ -2463,10 +2472,10 @@
         <v>3</v>
       </c>
       <c r="E70" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F70" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -2474,19 +2483,19 @@
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C71" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D71" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F71" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -2494,19 +2503,19 @@
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C72" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D72" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E72" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F72" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -2514,19 +2523,19 @@
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C73" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D73" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E73" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F73" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2534,16 +2543,16 @@
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C74" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D74" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E74" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F74" t="s">
         <v>63</v>
@@ -2554,16 +2563,16 @@
         <v>74</v>
       </c>
       <c r="B75" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C75" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D75" s="9">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E75" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F75" t="s">
         <v>65</v>
@@ -2574,16 +2583,16 @@
         <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C76" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D76" s="9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E76" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F76" t="s">
         <v>67</v>
@@ -2594,16 +2603,16 @@
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D77" s="9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E77" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F77" t="s">
         <v>69</v>
@@ -2614,7 +2623,7 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>19</v>
@@ -2623,7 +2632,7 @@
         <v>5</v>
       </c>
       <c r="E78" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F78" t="s">
         <v>71</v>
@@ -2634,16 +2643,16 @@
         <v>78</v>
       </c>
       <c r="B79" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D79" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E79" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F79" t="s">
         <v>73</v>
@@ -2654,19 +2663,19 @@
         <v>79</v>
       </c>
       <c r="B80" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D80" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E80" t="s">
-        <v>137</v>
+        <v>126</v>
       </c>
       <c r="F80" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2674,16 +2683,16 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D81" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E81" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F81" t="s">
         <v>78</v>
@@ -2694,16 +2703,16 @@
         <v>81</v>
       </c>
       <c r="B82" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="C82" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D82" s="9">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E82" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F82" t="s">
         <v>78</v>
@@ -2714,7 +2723,7 @@
         <v>82</v>
       </c>
       <c r="B83" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C83" s="8" t="s">
         <v>19</v>
@@ -2723,7 +2732,7 @@
         <v>5</v>
       </c>
       <c r="E83" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F83" t="s">
         <v>81</v>
@@ -2734,7 +2743,7 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C84" s="8" t="s">
         <v>19</v>
@@ -2743,7 +2752,7 @@
         <v>1</v>
       </c>
       <c r="E84" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F84" t="s">
         <v>83</v>
@@ -2754,7 +2763,7 @@
         <v>84</v>
       </c>
       <c r="B85" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C85" s="8" t="s">
         <v>19</v>
@@ -2763,7 +2772,7 @@
         <v>3</v>
       </c>
       <c r="E85" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F85" t="s">
         <v>85</v>
@@ -2774,7 +2783,7 @@
         <v>85</v>
       </c>
       <c r="B86" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C86" s="8" t="s">
         <v>19</v>
@@ -2783,7 +2792,7 @@
         <v>2</v>
       </c>
       <c r="E86" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F86" t="s">
         <v>87</v>
@@ -2794,16 +2803,16 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C87" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D87" s="9">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E87" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F87" t="s">
         <v>89</v>
@@ -2814,16 +2823,16 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C88" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D88" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E88" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F88" t="s">
         <v>78</v>
@@ -2834,7 +2843,7 @@
         <v>88</v>
       </c>
       <c r="B89" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="C89" s="8" t="s">
         <v>19</v>
@@ -2843,7 +2852,7 @@
         <v>3</v>
       </c>
       <c r="E89" t="s">
-        <v>137</v>
+        <v>157</v>
       </c>
       <c r="F89" t="s">
         <v>92</v>
@@ -2854,16 +2863,16 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="C90" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D90" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E90" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="F90" t="s">
         <v>94</v>
@@ -2874,16 +2883,16 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C91" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D91" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E91" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="F91" t="s">
         <v>96</v>
@@ -2894,16 +2903,16 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="C92" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D92" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E92" t="s">
-        <v>137</v>
+        <v>167</v>
       </c>
       <c r="F92" t="s">
         <v>78</v>
@@ -2914,13 +2923,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="C93" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D93" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E93" t="s">
         <v>167</v>
@@ -2934,7 +2943,7 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="C94" s="8" t="s">
         <v>19</v>
@@ -2954,7 +2963,7 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C95" s="8" t="s">
         <v>19</v>
@@ -2974,7 +2983,7 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C96" s="8" t="s">
         <v>19</v>
@@ -2986,7 +2995,7 @@
         <v>167</v>
       </c>
       <c r="F96" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -2994,7 +3003,7 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="C97" s="8" t="s">
         <v>19</v>
@@ -3006,7 +3015,7 @@
         <v>167</v>
       </c>
       <c r="F97" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -3014,19 +3023,19 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C98" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D98" s="9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E98" t="s">
         <v>167</v>
       </c>
       <c r="F98" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -3034,7 +3043,7 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C99" s="8" t="s">
         <v>19</v>
@@ -3046,7 +3055,7 @@
         <v>167</v>
       </c>
       <c r="F99" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -3054,19 +3063,19 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C100" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D100" s="9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E100" t="s">
         <v>167</v>
       </c>
       <c r="F100" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -3074,19 +3083,19 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="C101" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D101" s="9">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E101" t="s">
         <v>167</v>
       </c>
       <c r="F101" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -3094,19 +3103,19 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C102" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D102" s="9">
-        <v>388</v>
+        <v>151</v>
       </c>
       <c r="E102" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F102" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>